<commit_message>
Simplifica notebook da Atividade 3
- Codigo mais direto, menos comentario
- Tabelas salvas como curso_superior.xlsx, tecnologia.xlsx, educacao.xlsx
</commit_message>
<xml_diff>
--- a/Atividade 3/curso_superior.xlsx
+++ b/Atividade 3/curso_superior.xlsx
@@ -413,108 +413,123 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D6"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>regiao</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Homens</t>
+          <t>superior_total</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>Mulheres</t>
+          <t>superior_homens</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>superior_mulheres</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B2" t="inlineStr">
         <is>
           <t>Norte</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="C2" t="n">
         <v>1525166</v>
       </c>
-      <c r="C2" t="n">
+      <c r="D2" t="n">
         <v>590558</v>
       </c>
-      <c r="D2" t="n">
+      <c r="E2" t="n">
         <v>934609</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="inlineStr">
+      <c r="A3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B3" t="inlineStr">
         <is>
           <t>Nordeste</t>
         </is>
       </c>
-      <c r="B3" t="n">
+      <c r="C3" t="n">
         <v>4748933</v>
       </c>
-      <c r="C3" t="n">
+      <c r="D3" t="n">
         <v>1744994</v>
       </c>
-      <c r="D3" t="n">
+      <c r="E3" t="n">
         <v>3003939</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
+      <c r="A4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B4" t="inlineStr">
         <is>
           <t>Sudeste</t>
         </is>
       </c>
-      <c r="B4" t="n">
+      <c r="C4" t="n">
         <v>12828829</v>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="n">
         <v>5391638</v>
       </c>
-      <c r="D4" t="n">
+      <c r="E4" t="n">
         <v>7437191</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="inlineStr">
+      <c r="A5" t="n">
+        <v>4</v>
+      </c>
+      <c r="B5" t="inlineStr">
         <is>
           <t>Sul</t>
         </is>
       </c>
-      <c r="B5" t="n">
+      <c r="C5" t="n">
         <v>4338861</v>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="n">
         <v>1768855</v>
       </c>
-      <c r="D5" t="n">
+      <c r="E5" t="n">
         <v>2570005</v>
       </c>
     </row>
     <row r="6">
-      <c r="A6" t="inlineStr">
+      <c r="A6" t="n">
+        <v>5</v>
+      </c>
+      <c r="B6" t="inlineStr">
         <is>
           <t>Centro-Oeste</t>
         </is>
       </c>
-      <c r="B6" t="n">
+      <c r="C6" t="n">
         <v>2412502</v>
       </c>
-      <c r="C6" t="n">
+      <c r="D6" t="n">
         <v>982489</v>
       </c>
-      <c r="D6" t="n">
+      <c r="E6" t="n">
         <v>1430013</v>
       </c>
     </row>

</xml_diff>